<commit_message>
updated the title and added some text based on conference abstract.
</commit_message>
<xml_diff>
--- a/Data/craft learning.xlsx
+++ b/Data/craft learning.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25831"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FilesVC\HRAF-2022\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DBFF16E-96B4-43DF-89C9-E062B5FEBED8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E343949-5661-4764-B136-E929AB4728C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13276" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6561,7 +6561,7 @@
     <col min="17" max="17" width="14.33203125" customWidth="1"/>
     <col min="18" max="18" width="11.265625" customWidth="1"/>
     <col min="19" max="19" width="19.1328125" customWidth="1"/>
-    <col min="20" max="20" width="128.33203125" customWidth="1"/>
+    <col min="20" max="20" width="40" customWidth="1"/>
     <col min="21" max="21" width="11.9296875" customWidth="1"/>
     <col min="22" max="22" width="19.3984375" customWidth="1"/>
     <col min="23" max="23" width="16.86328125" customWidth="1"/>

</xml_diff>

<commit_message>
deleted all the insertfile in appendix.
</commit_message>
<xml_diff>
--- a/Data/craft learning.xlsx
+++ b/Data/craft learning.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25831"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FilesVC\HRAF-2022\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E343949-5661-4764-B136-E929AB4728C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0566F998-C732-400E-99DC-FA2074D818FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13276" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="craft learning" sheetId="1" r:id="rId1"/>
@@ -6546,6 +6546,7 @@
   <dimension ref="A1:Y520"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
+    <col min="1" max="1" width="12.73046875" customWidth="1"/>
     <col min="2" max="2" width="18.33203125" customWidth="1"/>
     <col min="4" max="4" width="26.86328125" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>

</xml_diff>